<commit_message>
Ajout contrôle fr-core-1 (#285)
* update

* update inv 906c94465ec93f1da252362532ba618a80ff600d
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-fr-core-patient-ins.xlsx
+++ b/main/ig/StructureDefinition-fr-core-patient-ins.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-23T10:39:10+00:00</t>
+    <t>2026-02-23T12:56:47+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -280,7 +280,7 @@
   </si>
   <si>
     <t>dom-2:If the resource is contained in another resource, it SHALL NOT contain nested Resources {contained.contained.empty()}
-dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}fr-core-1:If identityReliability status = 'VALI', then at least Patient.identifier[INS-NIR] or Patient.identifier[INS-NIA] or Patient.identifier[INS-NIR-TEST] or Patient.identifier[INS-NIR-DEMO] SHALL be present {(extension('https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-identity-reliability').extension('identityStatus').value.exists(code = 'VALI')) implies (identifier.where(system = 'urn:oid:1.2.250.1.213.1.4.8' and use = 'official').exists() or identifier.where(system = 'urn:oid:1.2.250.1.213.1.4.9' and use = 'official').exists() or identifier.where(system = 'urn:oid:1.2.250.1.213.1.4.10' and use = 'official').exists() or identifier.where(system = 'urn:oid:1.2.250.1.213.1.4.11' and use = 'official').exists())}fr-core-2:If identityReliability status = 'VALI', then only one identifier of type official SHALL be present {(extension('https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-identity-reliability').extension('identityStatus').value.exists(code = 'VALI')) implies (identifier.where(use = 'official').count() = 1)}fr-core-3:If identityReliability status = 'VALI', then the municipality of birth COG code cannot be 99999 because this code cannot be sent by the INSI online service. {(extension('https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-identity-reliability').extension('identityStatus').value.exists(code = 'VALI')) implies extension('http://hl7.org/fhir/StructureDefinition/patient-birthPlace').value.extension('https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-address-insee-code').value.code != '99999')}</t>
+dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}fr-core-1:If identityReliability status = 'VALI', then at least Patient.identifier[INS-NIR] or Patient.identifier[INS-NIA] or Patient.identifier[INS-NIR-TEST] or Patient.identifier[INS-NIR-DEMO] SHALL be present {(extension('https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-identity-reliability').extension('identityStatus').value.exists(code = 'VALI')) implies (identifier.where(system = 'urn:oid:1.2.250.1.213.1.4.8' and use = 'official' and type.coding.exists(code = 'INS-NIR')).exists() or identifier.where(system = 'urn:oid:1.2.250.1.213.1.4.9' and use = 'official').exists() or identifier.where(system = 'urn:oid:1.2.250.1.213.1.4.10' and use = 'official').exists() or identifier.where(system = 'urn:oid:1.2.250.1.213.1.4.11' and use = 'official').exists())}fr-core-2:If identityReliability status = 'VALI', then only one identifier of type official SHALL be present {(extension('https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-identity-reliability').extension('identityStatus').value.exists(code = 'VALI')) implies (identifier.where(use = 'official').count() = 1)}fr-core-3:If identityReliability status = 'VALI', then the municipality of birth COG code cannot be 99999 because this code cannot be sent by the INSI online service. {(extension('https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-identity-reliability').extension('identityStatus').value.exists(code = 'VALI')) implies extension('http://hl7.org/fhir/StructureDefinition/patient-birthPlace').value.extension('https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-address-insee-code').value.code != '99999'}</t>
   </si>
   <si>
     <t>Patient[classCode=PAT]</t>

</xml_diff>